<commit_message>
Add Excel workbook generator, screening merge script and empty template workbooks
scripts/build_workbooks.py builds screening, extraction (per-reviewer) and
appraisal workbooks from the 04_screening/05_extraction JSON templates:
dropdown-controlled codes, locked structure, text-formatted ID/gene-name
columns, in-sheet agreement and kappa formulas. scripts/merge_screening.py
merges two reviewer exports, computes agreement/kappa and PRISMA counts
(blank, never zero, until performed); selftest 27/27. templates_xlsx/
holds the regenerable empty workbooks. Team decision 2026-10-04: Excel
throughout, no Rayyan.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates_xlsx/appraisal_workbook.xlsx
+++ b/templates_xlsx/appraisal_workbook.xlsx
@@ -1286,7 +1286,7 @@
   <autoFilter ref="A1:I1"/>
   <dataValidations count="1">
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="tool_id" prompt="Tool from critical_appraisal_template tool_registry." type="list" errorStyle="stop">
-      <formula1>=ap_tool_id</formula1>
+      <formula1>ap_tool_id</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1366,13 +1366,13 @@
   <autoFilter ref="A1:I1"/>
   <dataValidations count="3">
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="tool_id" prompt="Tool from critical_appraisal_template tool_registry." type="list" errorStyle="stop">
-      <formula1>=ap_tool_id</formula1>
+      <formula1>ap_tool_id</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Not a listed code. For multi-valued fields separate codes with &quot;; &quot;. Press Yes to keep." promptTitle="appraiser_1_response" prompt="YES | NO | UNCLEAR | NA" type="list" errorStyle="warning">
-      <formula1>=ap_tool_response_normalized</formula1>
+      <formula1>ap_tool_response_normalized</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Not a listed code. For multi-valued fields separate codes with &quot;; &quot;. Press Yes to keep." promptTitle="appraiser_2_response" prompt="YES | NO | UNCLEAR | NA" type="list" errorStyle="warning">
-      <formula1>=ap_tool_response_normalized</formula1>
+      <formula1>ap_tool_response_normalized</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1458,13 +1458,13 @@
   <autoFilter ref="A1:J1"/>
   <dataValidations count="3">
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="tool_id" prompt="Tool from critical_appraisal_template tool_registry." type="list" errorStyle="stop">
-      <formula1>=ap_tool_id</formula1>
+      <formula1>ap_tool_id</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="response_normalized" prompt="YES | NO | UNCLEAR | NA" type="list" errorStyle="stop">
-      <formula1>=ap_tool_response_normalized</formula1>
+      <formula1>ap_tool_response_normalized</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="reporting_status" prompt="REPORTED | NR | CONFLICTING | NOT_APPLICABLE" type="list" errorStyle="stop">
-      <formula1>=ap_reporting_status</formula1>
+      <formula1>ap_reporting_status</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1694,37 +1694,37 @@
   <autoFilter ref="A1:AH1"/>
   <dataValidations count="11">
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
-      <formula1>=ap_precision_profile_status</formula1>
+      <formula1>ap_precision_profile_status</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
-      <formula1>=ap_precision_profile_status</formula1>
+      <formula1>ap_precision_profile_status</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
-      <formula1>=ap_precision_profile_status</formula1>
+      <formula1>ap_precision_profile_status</formula1>
     </dataValidation>
     <dataValidation sqref="N2:N1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
-      <formula1>=ap_precision_profile_status</formula1>
+      <formula1>ap_precision_profile_status</formula1>
     </dataValidation>
     <dataValidation sqref="Q2:Q1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
-      <formula1>=ap_precision_profile_status</formula1>
+      <formula1>ap_precision_profile_status</formula1>
     </dataValidation>
     <dataValidation sqref="S2:S1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="linkage_type" prompt="MOLECULAR_CONCORDANCE | CELL_COUNT_OR_SUBSET | EX_VIVO_FUNCTION | VACCINE_OR_ANTIBODY | SYMPTOM | PATHOGEN_CONFIRMED_INFECTION | OTHER | NR" type="list" errorStyle="stop">
-      <formula1>=ap_functional_linkage_type</formula1>
+      <formula1>ap_functional_linkage_type</formula1>
     </dataValidation>
     <dataValidation sqref="U2:U1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
-      <formula1>=ap_precision_profile_status</formula1>
+      <formula1>ap_precision_profile_status</formula1>
     </dataValidation>
     <dataValidation sqref="W2:W1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="validation_unit" prompt="PARTICIPANT | COHORT | SITE | TIME_PERIOD | OTHER | NR" type="list" errorStyle="stop">
-      <formula1>=ap_validation_unit</formula1>
+      <formula1>ap_validation_unit</formula1>
     </dataValidation>
     <dataValidation sqref="Y2:Y1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
-      <formula1>=ap_precision_profile_status</formula1>
+      <formula1>ap_precision_profile_status</formula1>
     </dataValidation>
     <dataValidation sqref="AA2:AA1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="use_tested" prompt="TESTED | NOT_TESTED | PROPOSED_ONLY | NR | UNCLEAR | NA" type="list" errorStyle="stop">
-      <formula1>=ap_decision_use_status</formula1>
+      <formula1>ap_decision_use_status</formula1>
     </dataValidation>
     <dataValidation sqref="AF2:AF1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
-      <formula1>=ap_precision_profile_status</formula1>
+      <formula1>ap_precision_profile_status</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2986,25 +2986,25 @@
   <autoFilter ref="A1:AB1"/>
   <dataValidations count="7">
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="eligibility_stratum" prompt="CORE_A | CORE_B | FRONTIER_PREPRINT | CONTEXT_ONLY | BOUNDARY_PILOT" type="list" errorStyle="stop">
-      <formula1>=ap_eligibility_stratum</formula1>
+      <formula1>ap_eligibility_stratum</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="core_appraisal_denominator" prompt="YES | NO | PENDING" type="list" errorStyle="stop">
-      <formula1>=ap_core_appraisal_denominator</formula1>
+      <formula1>ap_core_appraisal_denominator</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="publication_status" prompt="PEER_REVIEWED | PREPRINT | OTHER | UNCLEAR" type="list" errorStyle="stop">
-      <formula1>=ap_publication_status</formula1>
+      <formula1>ap_publication_status</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="tool_id" prompt="Tool from critical_appraisal_template tool_registry." type="list" errorStyle="stop">
-      <formula1>=ap_tool_id</formula1>
+      <formula1>ap_tool_id</formula1>
     </dataValidation>
     <dataValidation sqref="Q2:Q1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="analysis_phase_if_prediction_mo…" prompt="NOT_APPLICABLE | DEVELOPMENT | EVALUATION | BOTH" type="list" errorStyle="stop">
-      <formula1>=ap_prediction_model_phase</formula1>
+      <formula1>ap_prediction_model_phase</formula1>
     </dataValidation>
     <dataValidation sqref="R2:R1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="validation_type_if_prediction_m…" prompt="NOT_APPLICABLE | APPARENT | INTERNAL | EXTERNAL | MULTIPLE | NR" type="list" errorStyle="stop">
-      <formula1>=ap_prediction_validation_type</formula1>
+      <formula1>ap_prediction_validation_type</formula1>
     </dataValidation>
     <dataValidation sqref="X2:X1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="consensus_status" prompt="NOT_STARTED | DISCUSSED_RESOLVED | ADJUDICATOR_REQUIRED | ADJUDICATED" type="list" errorStyle="stop">
-      <formula1>=ap_consensus_status</formula1>
+      <formula1>ap_consensus_status</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3103,13 +3103,13 @@
   <autoFilter ref="A1:L1"/>
   <dataValidations count="3">
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="tool_id" prompt="Tool from critical_appraisal_template tool_registry." type="list" errorStyle="stop">
-      <formula1>=ap_only_JBI_RCT_CURRENT</formula1>
+      <formula1>ap_only_JBI_RCT_CURRENT</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="response_normalized" prompt="YES | NO | UNCLEAR | NA" type="list" errorStyle="stop">
-      <formula1>=ap_tool_response_normalized</formula1>
+      <formula1>ap_tool_response_normalized</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="reporting_status" prompt="REPORTED | NR | CONFLICTING | NOT_APPLICABLE" type="list" errorStyle="stop">
-      <formula1>=ap_reporting_status</formula1>
+      <formula1>ap_reporting_status</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3208,13 +3208,13 @@
   <autoFilter ref="A1:L1"/>
   <dataValidations count="3">
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="tool_id" prompt="Tool from critical_appraisal_template tool_registry." type="list" errorStyle="stop">
-      <formula1>=ap_only_JBI_QUASI_EXPERIMENTAL_CURRENT</formula1>
+      <formula1>ap_only_JBI_QUASI_EXPERIMENTAL_CURRENT</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="response_normalized" prompt="YES | NO | UNCLEAR | NA" type="list" errorStyle="stop">
-      <formula1>=ap_tool_response_normalized</formula1>
+      <formula1>ap_tool_response_normalized</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="reporting_status" prompt="REPORTED | NR | CONFLICTING | NOT_APPLICABLE" type="list" errorStyle="stop">
-      <formula1>=ap_reporting_status</formula1>
+      <formula1>ap_reporting_status</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3313,13 +3313,13 @@
   <autoFilter ref="A1:L1"/>
   <dataValidations count="3">
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="tool_id" prompt="Tool from critical_appraisal_template tool_registry." type="list" errorStyle="stop">
-      <formula1>=ap_only_JBI_COHORT_CURRENT</formula1>
+      <formula1>ap_only_JBI_COHORT_CURRENT</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="response_normalized" prompt="YES | NO | UNCLEAR | NA" type="list" errorStyle="stop">
-      <formula1>=ap_tool_response_normalized</formula1>
+      <formula1>ap_tool_response_normalized</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="reporting_status" prompt="REPORTED | NR | CONFLICTING | NOT_APPLICABLE" type="list" errorStyle="stop">
-      <formula1>=ap_reporting_status</formula1>
+      <formula1>ap_reporting_status</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3418,13 +3418,13 @@
   <autoFilter ref="A1:L1"/>
   <dataValidations count="3">
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="tool_id" prompt="Tool from critical_appraisal_template tool_registry." type="list" errorStyle="stop">
-      <formula1>=ap_only_JBI_ANALYTICAL_CROSS_SECTIONAL_CURRENT</formula1>
+      <formula1>ap_only_JBI_ANALYTICAL_CROSS_SECTIONAL_CURRENT</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="response_normalized" prompt="YES | NO | UNCLEAR | NA" type="list" errorStyle="stop">
-      <formula1>=ap_tool_response_normalized</formula1>
+      <formula1>ap_tool_response_normalized</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="reporting_status" prompt="REPORTED | NR | CONFLICTING | NOT_APPLICABLE" type="list" errorStyle="stop">
-      <formula1>=ap_reporting_status</formula1>
+      <formula1>ap_reporting_status</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3523,13 +3523,13 @@
   <autoFilter ref="A1:L1"/>
   <dataValidations count="3">
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="tool_id" prompt="Tool from critical_appraisal_template tool_registry." type="list" errorStyle="stop">
-      <formula1>=ap_only_JBI_CASE_CONTROL_CURRENT</formula1>
+      <formula1>ap_only_JBI_CASE_CONTROL_CURRENT</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="response_normalized" prompt="YES | NO | UNCLEAR | NA" type="list" errorStyle="stop">
-      <formula1>=ap_tool_response_normalized</formula1>
+      <formula1>ap_tool_response_normalized</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="reporting_status" prompt="REPORTED | NR | CONFLICTING | NOT_APPLICABLE" type="list" errorStyle="stop">
-      <formula1>=ap_reporting_status</formula1>
+      <formula1>ap_reporting_status</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3628,13 +3628,13 @@
   <autoFilter ref="A1:L1"/>
   <dataValidations count="3">
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="tool_id" prompt="Tool from critical_appraisal_template tool_registry." type="list" errorStyle="stop">
-      <formula1>=ap_only_JBI_DTA_CURRENT</formula1>
+      <formula1>ap_only_JBI_DTA_CURRENT</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="response_normalized" prompt="YES | NO | UNCLEAR | NA" type="list" errorStyle="stop">
-      <formula1>=ap_tool_response_normalized</formula1>
+      <formula1>ap_tool_response_normalized</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="reporting_status" prompt="REPORTED | NR | CONFLICTING | NOT_APPLICABLE" type="list" errorStyle="stop">
-      <formula1>=ap_reporting_status</formula1>
+      <formula1>ap_reporting_status</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3733,13 +3733,13 @@
   <autoFilter ref="A1:L1"/>
   <dataValidations count="3">
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="tool_id" prompt="Tool from critical_appraisal_template tool_registry." type="list" errorStyle="stop">
-      <formula1>=ap_only_PROBAST_AI_2025</formula1>
+      <formula1>ap_only_PROBAST_AI_2025</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="response_normalized" prompt="YES | NO | UNCLEAR | NA" type="list" errorStyle="stop">
-      <formula1>=ap_tool_response_normalized</formula1>
+      <formula1>ap_tool_response_normalized</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="reporting_status" prompt="REPORTED | NR | CONFLICTING | NOT_APPLICABLE" type="list" errorStyle="stop">
-      <formula1>=ap_reporting_status</formula1>
+      <formula1>ap_reporting_status</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
v3: extraction data model and synthesis plan aligned to the open-window organising construct
data_dictionary 3.0: marker_family, author_window_interpretation,
within_organising_window, exercise_duration/intensity, age_range,
adult_stratum_separable, older_adult_subgroup; one time-bin list
(pre_exercise_baseline ... 24h_to_72h_inclusive = within window, gt72h =
outside-window recovery); one Core A / Support B vocabulary; evidence-state
crosswalk; 35 undefined columns defined; duplicate codes removed;
extraction_template synced field-for-field (0 sync failures).
evidence_map_spec/synthesis_plan: figure 1 open-window time x compartment/
marker family, figure 2 per-marker validation-readiness map, prohibited
inference "adjudicates whether an open window exists". Blueprint: v3 titles,
positioning, GitHub+Zenodo, AI disclosure in Methods and Acknowledgments.
Workbooks regenerated (0 template issues). AI-use log updated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates_xlsx/appraisal_workbook.xlsx
+++ b/templates_xlsx/appraisal_workbook.xlsx
@@ -27,7 +27,7 @@
     <definedName name="ap_tool_response_normalized">'codes'!$A$2:$A$5</definedName>
     <definedName name="ap_reporting_status">'codes'!$C$2:$C$5</definedName>
     <definedName name="ap_precision_profile_status">'codes'!$E$2:$E$5</definedName>
-    <definedName name="ap_eligibility_stratum">'codes'!$G$2:$G$6</definedName>
+    <definedName name="ap_eligibility_stratum">'codes'!$G$2:$G$7</definedName>
     <definedName name="ap_core_appraisal_denominator">'codes'!$I$2:$I$4</definedName>
     <definedName name="ap_publication_status">'codes'!$K$2:$K$5</definedName>
     <definedName name="ap_prediction_model_phase">'codes'!$M$2:$M$5</definedName>
@@ -36,15 +36,16 @@
     <definedName name="ap_functional_linkage_type">'codes'!$S$2:$S$9</definedName>
     <definedName name="ap_validation_unit">'codes'!$U$2:$U$7</definedName>
     <definedName name="ap_decision_use_status">'codes'!$W$2:$W$7</definedName>
-    <definedName name="ap_tool_id">'codes'!$Y$2:$Y$8</definedName>
-    <definedName name="ap_tool_id_table">'codes'!$Y$2:$Z$8</definedName>
-    <definedName name="ap_only_JBI_RCT_CURRENT">'codes'!$AB$2:$AB$2</definedName>
-    <definedName name="ap_only_JBI_QUASI_EXPERIMENTAL_CURRENT">'codes'!$AD$2:$AD$2</definedName>
-    <definedName name="ap_only_JBI_COHORT_CURRENT">'codes'!$AF$2:$AF$2</definedName>
-    <definedName name="ap_only_JBI_ANALYTICAL_CROSS_SECTIONAL_CURRENT">'codes'!$AH$2:$AH$2</definedName>
-    <definedName name="ap_only_JBI_CASE_CONTROL_CURRENT">'codes'!$AJ$2:$AJ$2</definedName>
-    <definedName name="ap_only_JBI_DTA_CURRENT">'codes'!$AL$2:$AL$2</definedName>
-    <definedName name="ap_only_PROBAST_AI_2025">'codes'!$AN$2:$AN$2</definedName>
+    <definedName name="ap_window_coverage">'codes'!$Y$2:$Y$6</definedName>
+    <definedName name="ap_tool_id">'codes'!$AA$2:$AA$8</definedName>
+    <definedName name="ap_tool_id_table">'codes'!$AA$2:$AB$8</definedName>
+    <definedName name="ap_only_JBI_RCT_CURRENT">'codes'!$AD$2:$AD$2</definedName>
+    <definedName name="ap_only_JBI_QUASI_EXPERIMENTAL_CURRENT">'codes'!$AF$2:$AF$2</definedName>
+    <definedName name="ap_only_JBI_COHORT_CURRENT">'codes'!$AH$2:$AH$2</definedName>
+    <definedName name="ap_only_JBI_ANALYTICAL_CROSS_SECTIONAL_CURRENT">'codes'!$AJ$2:$AJ$2</definedName>
+    <definedName name="ap_only_JBI_CASE_CONTROL_CURRENT">'codes'!$AL$2:$AL$2</definedName>
+    <definedName name="ap_only_JBI_DTA_CURRENT">'codes'!$AN$2:$AN$2</definedName>
+    <definedName name="ap_only_PROBAST_AI_2025">'codes'!$AP$2:$AP$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'appraisal_records'!$A$1:$AB$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'JBI_RCT_CURRENT'!$A$1:$L$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'JBI_QUASI_EXPERIMENTAL_CURRENT'!$A$1:$L$1</definedName>
@@ -56,7 +57,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'official_tool_outputs'!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'initial_disagreements'!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'consensus_items'!$A$1:$J$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'precision_profile'!$A$1:$AH$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'precision_profile'!$A$1:$AJ$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -217,7 +218,7 @@
   <commentList>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Values: CORE_A | CORE_B | FRONTIER_PREPRINT | CONTEXT_ONLY | BOUNDARY_PILOT (status_codes.eligibility_stratum). Keep any source instrument's exact answer label in tool_response_verbatim. No report information is usually tool_response_normalized=UNCLEAR and reporting_status=NR, not NO. NR means not reported; it does not mean failed or absent. NA requires a rationale. Status codes are descriptive, not points or a scale.</t>
+        <t>Values: A_core_acute | B_support_repeated_bouts | background | uncertain | FRONTIER_PREPRINT | BOUNDARY_PILOT (status_codes.eligibility_stratum). Keep any source instrument's exact answer label in tool_response_verbatim. No report information is usually tool_response_normalized=UNCLEAR and reporting_status=NR, not NO. NR means not reported; it does not mean failed or absent. NA requires a rationale. Status codes are descriptive, not points or a scale.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
@@ -315,47 +316,52 @@
         <t>Values: EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE (status_codes.precision_profile_status). Keep any source instrument's exact answer label in tool_response_verbatim. No report information is usually tool_response_normalized=UNCLEAR and reporting_status=NR, not NO. NR means not reported; it does not mean failed or absent. NA requires a rationale. Status codes are descriptive, not points or a scale.</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Values: WITHIN_WINDOW_ONLY | WITHIN_AND_OUTSIDE_WINDOW | OUTSIDE_WINDOW_ONLY | NR | UNCLEAR (status_codes.window_coverage). Keep any source instrument's exact answer label in tool_response_verbatim. No report information is usually tool_response_normalized=UNCLEAR and reporting_status=NR, not NO. NR means not reported; it does not mean failed or absent. NA requires a rationale. Status codes are descriptive, not points or a scale.</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <t>Values: EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE (status_codes.precision_profile_status). Keep any source instrument's exact answer label in tool_response_verbatim. No report information is usually tool_response_normalized=UNCLEAR and reporting_status=NR, not NO. NR means not reported; it does not mean failed or absent. NA requires a rationale. Status codes are descriptive, not points or a scale.</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <t>Values: EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE (status_codes.precision_profile_status). Keep any source instrument's exact answer label in tool_response_verbatim. No report information is usually tool_response_normalized=UNCLEAR and reporting_status=NR, not NO. NR means not reported; it does not mean failed or absent. NA requires a rationale. Status codes are descriptive, not points or a scale.</t>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
+    <comment ref="S1" authorId="0" shapeId="0">
       <text>
         <t>Values: EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE (status_codes.precision_profile_status). Keep any source instrument's exact answer label in tool_response_verbatim. No report information is usually tool_response_normalized=UNCLEAR and reporting_status=NR, not NO. NR means not reported; it does not mean failed or absent. NA requires a rationale. Status codes are descriptive, not points or a scale.</t>
       </text>
     </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
+    <comment ref="U1" authorId="0" shapeId="0">
       <text>
         <t>Values: MOLECULAR_CONCORDANCE | CELL_COUNT_OR_SUBSET | EX_VIVO_FUNCTION | VACCINE_OR_ANTIBODY | SYMPTOM | PATHOGEN_CONFIRMED_INFECTION | OTHER | NR (status_codes.functional_linkage_type). Keep any source instrument's exact answer label in tool_response_verbatim. No report information is usually tool_response_normalized=UNCLEAR and reporting_status=NR, not NO. NR means not reported; it does not mean failed or absent. NA requires a rationale. Status codes are descriptive, not points or a scale.</t>
       </text>
     </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
+    <comment ref="W1" authorId="0" shapeId="0">
       <text>
         <t>Values: EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE (status_codes.precision_profile_status). Keep any source instrument's exact answer label in tool_response_verbatim. No report information is usually tool_response_normalized=UNCLEAR and reporting_status=NR, not NO. NR means not reported; it does not mean failed or absent. NA requires a rationale. Status codes are descriptive, not points or a scale.</t>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
+    <comment ref="Y1" authorId="0" shapeId="0">
       <text>
         <t>Values: PARTICIPANT | COHORT | SITE | TIME_PERIOD | OTHER | NR (status_codes.validation_unit). Keep any source instrument's exact answer label in tool_response_verbatim. No report information is usually tool_response_normalized=UNCLEAR and reporting_status=NR, not NO. NR means not reported; it does not mean failed or absent. NA requires a rationale. Status codes are descriptive, not points or a scale.</t>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
+    <comment ref="AA1" authorId="0" shapeId="0">
       <text>
         <t>Values: EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE (status_codes.precision_profile_status). Keep any source instrument's exact answer label in tool_response_verbatim. No report information is usually tool_response_normalized=UNCLEAR and reporting_status=NR, not NO. NR means not reported; it does not mean failed or absent. NA requires a rationale. Status codes are descriptive, not points or a scale.</t>
       </text>
     </comment>
-    <comment ref="AA1" authorId="0" shapeId="0">
+    <comment ref="AC1" authorId="0" shapeId="0">
       <text>
         <t>Values: TESTED | NOT_TESTED | PROPOSED_ONLY | NR | UNCLEAR | NA (status_codes.decision_use_status). Keep any source instrument's exact answer label in tool_response_verbatim. No report information is usually tool_response_normalized=UNCLEAR and reporting_status=NR, not NO. NR means not reported; it does not mean failed or absent. NA requires a rationale. Status codes are descriptive, not points or a scale.</t>
       </text>
     </comment>
-    <comment ref="AF1" authorId="0" shapeId="0">
+    <comment ref="AH1" authorId="0" shapeId="0">
       <text>
         <t>Values: EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE (status_codes.precision_profile_status). Keep any source instrument's exact answer label in tool_response_verbatim. No report information is usually tool_response_normalized=UNCLEAR and reporting_status=NR, not NO. NR means not reported; it does not mean failed or absent. NA requires a rationale. Status codes are descriptive, not points or a scale.</t>
       </text>
@@ -426,6 +432,11 @@
       </text>
     </comment>
     <comment ref="W1" authorId="0" shapeId="0">
+      <text>
+        <t>Keep any source instrument's exact answer label in tool_response_verbatim. No report information is usually tool_response_normalized=UNCLEAR and reporting_status=NR, not NO. NR means not reported; it does not mean failed or absent. NA requires a rationale. Status codes are descriptive, not points or a scale.</t>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
       <text>
         <t>Keep any source instrument's exact answer label in tool_response_verbatim. No report information is usually tool_response_normalized=UNCLEAR and reporting_status=NR, not NO. NR means not reported; it does not mean failed or absent. NA requires a rationale. Status codes are descriptive, not points or a scale.</t>
       </text>
@@ -979,7 +990,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1022,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>template_version=1.0.0; protocol_version=2.0; accessed_on=2026-10-02; sha256=623b5c1abdbbc35a…</t>
+          <t>template_version=1.0.0; protocol_version=3.0; accessed_on=2026-10-02; sha256=0acfd89611441ef7…</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1034,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>v2.0 working protocol, 2026-10-02; sha256=a7e4ced20c2db0b2…</t>
+          <t>v3.0 (draft for team freeze) - 4 October 2026 (`01_protocol/v3_design_contract.txt`); tool sources checked 2026-10-02; sha256=dc32373c28c50e02…</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1049,7 @@
     <row r="15">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Descriptive design-appropriate critical appraisal and a separate project-defined precision/assay profile. No composite score, rank, exclusion threshold, or GRADE certainty rating.</t>
+          <t>Descriptive design-appropriate critical appraisal and a separate project-defined precision/assay profile. No composite score, rank, exclusion threshold, or GRADE certainty rating. The precision profile feeds the validation-readiness map (see the validation-readiness map definition in this file; contract 8.3e). Validation-readiness map: a per-marker, domain-by-domain descriptive profile across the seven precision domains; not a score, ranking, grade or development ladder.</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1114,7 @@
     <row r="26">
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>precision_profile_note: Dimensions are reported separately and are not a validated scale, composite score, or ladder. Independent validation and tested decision use are recorded as separate facets within one protocol domain.</t>
+          <t>precision_profile_note: Dimensions are reported separately and are not a validated scale, composite score, or ladder; they feed the validation-readiness map (see the validation-readiness map definition in this file; contract 8.3e). Independent validation and tested decision use are recorded as separate facets within one protocol domain. temporal_validity.window_coverage summarises sample positions relative to the 0-72 h organising window (outside-window recovery samples are charted, never excluded); window_bins_covered lists the data_dictionary.json time_bin IDs covered, "; "-separated.</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1142,7 @@
     <row r="30">
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>process.reporting: Preserve both initial appraisals and consensus; summarize concerns descriptively by design without total score, ranking, appraisal-based exclusion, GRADE, or clinical recommendations.</t>
+          <t>process.reporting: Preserve both initial appraisals and consensus; summarize concerns descriptively by design without total score, ranking, appraisal-based exclusion, GRADE, or clinical recommendations. Precision-profile results enter only the validation-readiness map (see the validation-readiness map definition in this file; contract 8.3e).</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH1"/>
+  <dimension ref="A1:AJ1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="5" min="1" max="1"/>
@@ -1515,6 +1526,8 @@
     <col width="18" customWidth="1" style="5" min="32" max="32"/>
     <col width="18" customWidth="1" style="5" min="33" max="33"/>
     <col width="18" customWidth="1" style="5" min="34" max="34"/>
+    <col width="18" customWidth="1" style="5" min="35" max="35"/>
+    <col width="18" customWidth="1" style="5" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1565,125 +1578,135 @@
       </c>
       <c r="J1" s="6" t="inlineStr">
         <is>
+          <t>temporal_validity.window_coverage</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>temporal_validity.window_bins_covered</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
           <t>temporal_validity.evidence_locator</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>immune_specificity.status</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>immune_specificity.evidence_note</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>immune_specificity.evidence_locator</t>
         </is>
       </c>
-      <c r="N1" s="6" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>individualization.status</t>
         </is>
       </c>
-      <c r="O1" s="6" t="inlineStr">
+      <c r="Q1" s="6" t="inlineStr">
         <is>
           <t>individualization.evidence_note</t>
         </is>
       </c>
-      <c r="P1" s="6" t="inlineStr">
+      <c r="R1" s="6" t="inlineStr">
         <is>
           <t>individualization.evidence_locator</t>
         </is>
       </c>
-      <c r="Q1" s="6" t="inlineStr">
+      <c r="S1" s="6" t="inlineStr">
         <is>
           <t>functional_clinical_linkage.status</t>
         </is>
       </c>
-      <c r="R1" s="6" t="inlineStr">
+      <c r="T1" s="6" t="inlineStr">
         <is>
           <t>functional_clinical_linkage.evidence_note</t>
         </is>
       </c>
-      <c r="S1" s="6" t="inlineStr">
+      <c r="U1" s="6" t="inlineStr">
         <is>
           <t>functional_clinical_linkage.linkage_type</t>
         </is>
       </c>
-      <c r="T1" s="6" t="inlineStr">
+      <c r="V1" s="6" t="inlineStr">
         <is>
           <t>functional_clinical_linkage.evidence_locator</t>
         </is>
       </c>
-      <c r="U1" s="6" t="inlineStr">
+      <c r="W1" s="6" t="inlineStr">
         <is>
           <t>independent_validation_and_use.independent_validation.status</t>
         </is>
       </c>
-      <c r="V1" s="6" t="inlineStr">
+      <c r="X1" s="6" t="inlineStr">
         <is>
           <t>independent_validation_and_use.independent_validation.evidence_note</t>
         </is>
       </c>
-      <c r="W1" s="6" t="inlineStr">
+      <c r="Y1" s="6" t="inlineStr">
         <is>
           <t>independent_validation_and_use.independent_validation.validation_unit</t>
         </is>
       </c>
-      <c r="X1" s="6" t="inlineStr">
+      <c r="Z1" s="6" t="inlineStr">
         <is>
           <t>independent_validation_and_use.independent_validation.evidence_locator</t>
         </is>
       </c>
-      <c r="Y1" s="6" t="inlineStr">
+      <c r="AA1" s="6" t="inlineStr">
         <is>
           <t>independent_validation_and_use.decision_use_evidence.status</t>
         </is>
       </c>
-      <c r="Z1" s="6" t="inlineStr">
+      <c r="AB1" s="6" t="inlineStr">
         <is>
           <t>independent_validation_and_use.decision_use_evidence.intended_or_author_stated_use</t>
         </is>
       </c>
-      <c r="AA1" s="6" t="inlineStr">
+      <c r="AC1" s="6" t="inlineStr">
         <is>
           <t>independent_validation_and_use.decision_use_evidence.use_tested</t>
         </is>
       </c>
-      <c r="AB1" s="6" t="inlineStr">
+      <c r="AD1" s="6" t="inlineStr">
         <is>
           <t>independent_validation_and_use.decision_use_evidence.decision_context</t>
         </is>
       </c>
-      <c r="AC1" s="6" t="inlineStr">
+      <c r="AE1" s="6" t="inlineStr">
         <is>
           <t>independent_validation_and_use.decision_use_evidence.threshold_or_action</t>
         </is>
       </c>
-      <c r="AD1" s="6" t="inlineStr">
+      <c r="AF1" s="6" t="inlineStr">
         <is>
           <t>independent_validation_and_use.decision_use_evidence.implementation_or_decision_impact</t>
         </is>
       </c>
-      <c r="AE1" s="6" t="inlineStr">
+      <c r="AG1" s="6" t="inlineStr">
         <is>
           <t>independent_validation_and_use.decision_use_evidence.evidence_locator</t>
         </is>
       </c>
-      <c r="AF1" s="6" t="inlineStr">
+      <c r="AH1" s="6" t="inlineStr">
         <is>
           <t>feasibility.status</t>
         </is>
       </c>
-      <c r="AG1" s="6" t="inlineStr">
+      <c r="AI1" s="6" t="inlineStr">
         <is>
           <t>feasibility.evidence_note</t>
         </is>
       </c>
-      <c r="AH1" s="6" t="inlineStr">
+      <c r="AJ1" s="6" t="inlineStr">
         <is>
           <t>feasibility.evidence_locator</t>
         </is>
@@ -1691,39 +1714,42 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="0" sort="0"/>
-  <autoFilter ref="A1:AH1"/>
-  <dataValidations count="11">
+  <autoFilter ref="A1:AJ1"/>
+  <dataValidations count="12">
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
       <formula1>ap_precision_profile_status</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
       <formula1>ap_precision_profile_status</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
+    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="window_coverage" prompt="WITHIN_WINDOW_ONLY | WITHIN_AND_OUTSIDE_WINDOW | OUTSIDE_WINDOW_ONLY | NR | UNCLEAR" type="list" errorStyle="stop">
+      <formula1>ap_window_coverage</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
       <formula1>ap_precision_profile_status</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
+    <dataValidation sqref="P2:P1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
       <formula1>ap_precision_profile_status</formula1>
     </dataValidation>
-    <dataValidation sqref="Q2:Q1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
+    <dataValidation sqref="S2:S1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
       <formula1>ap_precision_profile_status</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="linkage_type" prompt="MOLECULAR_CONCORDANCE | CELL_COUNT_OR_SUBSET | EX_VIVO_FUNCTION | VACCINE_OR_ANTIBODY | SYMPTOM | PATHOGEN_CONFIRMED_INFECTION | OTHER | NR" type="list" errorStyle="stop">
+    <dataValidation sqref="U2:U1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="linkage_type" prompt="MOLECULAR_CONCORDANCE | CELL_COUNT_OR_SUBSET | EX_VIVO_FUNCTION | VACCINE_OR_ANTIBODY | SYMPTOM | PATHOGEN_CONFIRMED_INFECTION | OTHER | NR" type="list" errorStyle="stop">
       <formula1>ap_functional_linkage_type</formula1>
     </dataValidation>
-    <dataValidation sqref="U2:U1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
+    <dataValidation sqref="W2:W1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
       <formula1>ap_precision_profile_status</formula1>
     </dataValidation>
-    <dataValidation sqref="W2:W1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="validation_unit" prompt="PARTICIPANT | COHORT | SITE | TIME_PERIOD | OTHER | NR" type="list" errorStyle="stop">
+    <dataValidation sqref="Y2:Y1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="validation_unit" prompt="PARTICIPANT | COHORT | SITE | TIME_PERIOD | OTHER | NR" type="list" errorStyle="stop">
       <formula1>ap_validation_unit</formula1>
     </dataValidation>
-    <dataValidation sqref="Y2:Y1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
+    <dataValidation sqref="AA2:AA1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
       <formula1>ap_precision_profile_status</formula1>
     </dataValidation>
-    <dataValidation sqref="AA2:AA1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="use_tested" prompt="TESTED | NOT_TESTED | PROPOSED_ONLY | NR | UNCLEAR | NA" type="list" errorStyle="stop">
+    <dataValidation sqref="AC2:AC1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="use_tested" prompt="TESTED | NOT_TESTED | PROPOSED_ONLY | NR | UNCLEAR | NA" type="list" errorStyle="stop">
       <formula1>ap_decision_use_status</formula1>
     </dataValidation>
-    <dataValidation sqref="AF2:AF1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
+    <dataValidation sqref="AH2:AH1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="status" prompt="EVIDENCE_REPORTED | NOT_REPORTED | UNCLEAR | NOT_APPLICABLE" type="list" errorStyle="stop">
       <formula1>ap_precision_profile_status</formula1>
     </dataValidation>
   </dataValidations>
@@ -1979,7 +2005,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Habitual-exercise-only cross-sectional evidence is background under v2 and excluded from the core A/B appraisal denominator unless separately labeled as contextual.</t>
+          <t>Habitual-exercise-only cross-sectional evidence is background under v3 (contract 2.5, unchanged from v2) and excluded from the Core A / Support B appraisal denominator unless separately labeled as background.</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr"/>
@@ -2249,7 +2275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN9"/>
+  <dimension ref="A1:AP9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2265,14 +2291,15 @@
     <col width="28" customWidth="1" min="21" max="21"/>
     <col width="28" customWidth="1" min="23" max="23"/>
     <col width="28" customWidth="1" min="25" max="25"/>
-    <col width="48" customWidth="1" min="26" max="26"/>
-    <col width="28" customWidth="1" min="28" max="28"/>
+    <col width="28" customWidth="1" min="27" max="27"/>
+    <col width="48" customWidth="1" min="28" max="28"/>
     <col width="28" customWidth="1" min="30" max="30"/>
     <col width="28" customWidth="1" min="32" max="32"/>
     <col width="28" customWidth="1" min="34" max="34"/>
     <col width="28" customWidth="1" min="36" max="36"/>
     <col width="28" customWidth="1" min="38" max="38"/>
     <col width="28" customWidth="1" min="40" max="40"/>
+    <col width="28" customWidth="1" min="42" max="42"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2338,45 +2365,50 @@
       </c>
       <c r="Y1" s="6" t="inlineStr">
         <is>
+          <t>window_coverage</t>
+        </is>
+      </c>
+      <c r="AA1" s="6" t="inlineStr">
+        <is>
           <t>tool_id (tool_registry)</t>
         </is>
       </c>
-      <c r="Z1" s="6" t="inlineStr">
+      <c r="AB1" s="6" t="inlineStr">
         <is>
           <t>tool_name</t>
         </is>
       </c>
-      <c r="AB1" s="6" t="inlineStr">
+      <c r="AD1" s="6" t="inlineStr">
         <is>
           <t>tool_id for sheet JBI_RCT_CURRENT</t>
         </is>
       </c>
-      <c r="AD1" s="6" t="inlineStr">
+      <c r="AF1" s="6" t="inlineStr">
         <is>
           <t>tool_id for sheet JBI_QUASI_EXPERIMENTAL_CURRENT</t>
         </is>
       </c>
-      <c r="AF1" s="6" t="inlineStr">
+      <c r="AH1" s="6" t="inlineStr">
         <is>
           <t>tool_id for sheet JBI_COHORT_CURRENT</t>
         </is>
       </c>
-      <c r="AH1" s="6" t="inlineStr">
+      <c r="AJ1" s="6" t="inlineStr">
         <is>
           <t>tool_id for sheet JBI_ANALYTICAL_CROSS_SECTIONAL</t>
         </is>
       </c>
-      <c r="AJ1" s="6" t="inlineStr">
+      <c r="AL1" s="6" t="inlineStr">
         <is>
           <t>tool_id for sheet JBI_CASE_CONTROL_CURRENT</t>
         </is>
       </c>
-      <c r="AL1" s="6" t="inlineStr">
+      <c r="AN1" s="6" t="inlineStr">
         <is>
           <t>tool_id for sheet JBI_DTA_CURRENT</t>
         </is>
       </c>
-      <c r="AN1" s="6" t="inlineStr">
+      <c r="AP1" s="6" t="inlineStr">
         <is>
           <t>tool_id for sheet PROBAST_AI_2025</t>
         </is>
@@ -2400,7 +2432,7 @@
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>CORE_A</t>
+          <t>A_core_acute</t>
         </is>
       </c>
       <c r="I2" s="8" t="inlineStr">
@@ -2445,45 +2477,50 @@
       </c>
       <c r="Y2" s="8" t="inlineStr">
         <is>
+          <t>WITHIN_WINDOW_ONLY</t>
+        </is>
+      </c>
+      <c r="AA2" s="8" t="inlineStr">
+        <is>
           <t>JBI_RCT_CURRENT</t>
         </is>
       </c>
-      <c r="Z2" s="8" t="inlineStr">
+      <c r="AB2" s="8" t="inlineStr">
         <is>
           <t>JBI randomized controlled trials checklist</t>
         </is>
       </c>
-      <c r="AB2" s="8" t="inlineStr">
+      <c r="AD2" s="8" t="inlineStr">
         <is>
           <t>JBI_RCT_CURRENT</t>
         </is>
       </c>
-      <c r="AD2" s="8" t="inlineStr">
+      <c r="AF2" s="8" t="inlineStr">
         <is>
           <t>JBI_QUASI_EXPERIMENTAL_CURRENT</t>
         </is>
       </c>
-      <c r="AF2" s="8" t="inlineStr">
+      <c r="AH2" s="8" t="inlineStr">
         <is>
           <t>JBI_COHORT_CURRENT</t>
         </is>
       </c>
-      <c r="AH2" s="8" t="inlineStr">
+      <c r="AJ2" s="8" t="inlineStr">
         <is>
           <t>JBI_ANALYTICAL_CROSS_SECTIONAL_CURRENT</t>
         </is>
       </c>
-      <c r="AJ2" s="8" t="inlineStr">
+      <c r="AL2" s="8" t="inlineStr">
         <is>
           <t>JBI_CASE_CONTROL_CURRENT</t>
         </is>
       </c>
-      <c r="AL2" s="8" t="inlineStr">
+      <c r="AN2" s="8" t="inlineStr">
         <is>
           <t>JBI_DTA_CURRENT</t>
         </is>
       </c>
-      <c r="AN2" s="8" t="inlineStr">
+      <c r="AP2" s="8" t="inlineStr">
         <is>
           <t>PROBAST_AI_2025</t>
         </is>
@@ -2507,7 +2544,7 @@
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>CORE_B</t>
+          <t>B_support_repeated_bouts</t>
         </is>
       </c>
       <c r="I3" s="8" t="inlineStr">
@@ -2552,10 +2589,15 @@
       </c>
       <c r="Y3" s="8" t="inlineStr">
         <is>
+          <t>WITHIN_AND_OUTSIDE_WINDOW</t>
+        </is>
+      </c>
+      <c r="AA3" s="8" t="inlineStr">
+        <is>
           <t>JBI_QUASI_EXPERIMENTAL_CURRENT</t>
         </is>
       </c>
-      <c r="Z3" s="8" t="inlineStr">
+      <c r="AB3" s="8" t="inlineStr">
         <is>
           <t>JBI quasi-experimental studies checklist, revised</t>
         </is>
@@ -2579,7 +2621,7 @@
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>FRONTIER_PREPRINT</t>
+          <t>background</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr">
@@ -2624,10 +2666,15 @@
       </c>
       <c r="Y4" s="8" t="inlineStr">
         <is>
+          <t>OUTSIDE_WINDOW_ONLY</t>
+        </is>
+      </c>
+      <c r="AA4" s="8" t="inlineStr">
+        <is>
           <t>JBI_COHORT_CURRENT</t>
         </is>
       </c>
-      <c r="Z4" s="8" t="inlineStr">
+      <c r="AB4" s="8" t="inlineStr">
         <is>
           <t>JBI cohort studies checklist, revised</t>
         </is>
@@ -2651,7 +2698,7 @@
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>CONTEXT_ONLY</t>
+          <t>uncertain</t>
         </is>
       </c>
       <c r="K5" s="8" t="inlineStr">
@@ -2691,10 +2738,15 @@
       </c>
       <c r="Y5" s="8" t="inlineStr">
         <is>
+          <t>NR</t>
+        </is>
+      </c>
+      <c r="AA5" s="8" t="inlineStr">
+        <is>
           <t>JBI_ANALYTICAL_CROSS_SECTIONAL_CURRENT</t>
         </is>
       </c>
-      <c r="Z5" s="8" t="inlineStr">
+      <c r="AB5" s="8" t="inlineStr">
         <is>
           <t>JBI analytical cross-sectional studies risk-of-bias assessment, revised</t>
         </is>
@@ -2703,41 +2755,51 @@
     <row r="6">
       <c r="G6" s="8" t="inlineStr">
         <is>
+          <t>FRONTIER_PREPRINT</t>
+        </is>
+      </c>
+      <c r="O6" s="8" t="inlineStr">
+        <is>
+          <t>MULTIPLE</t>
+        </is>
+      </c>
+      <c r="S6" s="8" t="inlineStr">
+        <is>
+          <t>SYMPTOM</t>
+        </is>
+      </c>
+      <c r="U6" s="8" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="W6" s="8" t="inlineStr">
+        <is>
+          <t>UNCLEAR</t>
+        </is>
+      </c>
+      <c r="Y6" s="8" t="inlineStr">
+        <is>
+          <t>UNCLEAR</t>
+        </is>
+      </c>
+      <c r="AA6" s="8" t="inlineStr">
+        <is>
+          <t>JBI_CASE_CONTROL_CURRENT</t>
+        </is>
+      </c>
+      <c r="AB6" s="8" t="inlineStr">
+        <is>
+          <t>JBI case-control studies checklist</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="G7" s="8" t="inlineStr">
+        <is>
           <t>BOUNDARY_PILOT</t>
         </is>
       </c>
-      <c r="O6" s="8" t="inlineStr">
-        <is>
-          <t>MULTIPLE</t>
-        </is>
-      </c>
-      <c r="S6" s="8" t="inlineStr">
-        <is>
-          <t>SYMPTOM</t>
-        </is>
-      </c>
-      <c r="U6" s="8" t="inlineStr">
-        <is>
-          <t>OTHER</t>
-        </is>
-      </c>
-      <c r="W6" s="8" t="inlineStr">
-        <is>
-          <t>UNCLEAR</t>
-        </is>
-      </c>
-      <c r="Y6" s="8" t="inlineStr">
-        <is>
-          <t>JBI_CASE_CONTROL_CURRENT</t>
-        </is>
-      </c>
-      <c r="Z6" s="8" t="inlineStr">
-        <is>
-          <t>JBI case-control studies checklist</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
       <c r="O7" s="8" t="inlineStr">
         <is>
           <t>NR</t>
@@ -2758,12 +2820,12 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="Y7" s="8" t="inlineStr">
+      <c r="AA7" s="8" t="inlineStr">
         <is>
           <t>JBI_DTA_CURRENT</t>
         </is>
       </c>
-      <c r="Z7" s="8" t="inlineStr">
+      <c r="AB7" s="8" t="inlineStr">
         <is>
           <t>JBI diagnostic test accuracy studies checklist</t>
         </is>
@@ -2775,12 +2837,12 @@
           <t>OTHER</t>
         </is>
       </c>
-      <c r="Y8" s="8" t="inlineStr">
+      <c r="AA8" s="8" t="inlineStr">
         <is>
           <t>PROBAST_AI_2025</t>
         </is>
       </c>
-      <c r="Z8" s="8" t="inlineStr">
+      <c r="AB8" s="8" t="inlineStr">
         <is>
           <t>PROBAST+AI</t>
         </is>
@@ -2985,7 +3047,7 @@
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="0" sort="0"/>
   <autoFilter ref="A1:AB1"/>
   <dataValidations count="7">
-    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="eligibility_stratum" prompt="CORE_A | CORE_B | FRONTIER_PREPRINT | CONTEXT_ONLY | BOUNDARY_PILOT" type="list" errorStyle="stop">
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="eligibility_stratum" prompt="A_core_acute | B_support_repeated_bouts | background | uncertain | FRONTIER_PREPRINT | BOUNDARY_PILOT" type="list" errorStyle="stop">
       <formula1>ap_eligibility_stratum</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not in code list" error="Choose a value from the dropdown (codes sheet). Codes come from the JSON templates." promptTitle="core_appraisal_denominator" prompt="YES | NO | PENDING" type="list" errorStyle="stop">

</xml_diff>